<commit_message>
Change to single-group clustering instead of 2 levels
</commit_message>
<xml_diff>
--- a/output/cluster_review_edits.xlsx
+++ b/output/cluster_review_edits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilya/spatial-queries/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F652DCFF-CBEC-F04D-B1C3-D66CE8A15177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A4460B-3118-6749-82E5-D09FE017C545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="235">
   <si>
     <t>label</t>
   </si>
@@ -713,6 +713,18 @@
   </si>
   <si>
     <t>Generic factual queries</t>
+  </si>
+  <si>
+    <t>Distance and proximity</t>
+  </si>
+  <si>
+    <t>Occurrence</t>
+  </si>
+  <si>
+    <t>Temporal</t>
+  </si>
+  <si>
+    <t>group</t>
   </si>
 </sst>
 </file>
@@ -742,7 +754,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,6 +770,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -800,7 +818,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -813,6 +831,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1123,7 +1145,7 @@
     <col min="5" max="5" width="67.83203125" customWidth="1"/>
     <col min="6" max="6" width="23.83203125" customWidth="1"/>
     <col min="7" max="7" width="23.33203125" customWidth="1"/>
-    <col min="8" max="8" width="3.5" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="53.6640625" customWidth="1"/>
     <col min="10" max="10" width="37.33203125" customWidth="1"/>
   </cols>
@@ -1150,6 +1172,9 @@
       <c r="G1" s="2" t="s">
         <v>79</v>
       </c>
+      <c r="H1" s="6" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -1173,6 +1198,9 @@
       <c r="G2" t="s">
         <v>162</v>
       </c>
+      <c r="H2" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -1196,6 +1224,9 @@
       <c r="G3" t="s">
         <v>165</v>
       </c>
+      <c r="H3" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
@@ -1219,6 +1250,9 @@
       <c r="G4" t="s">
         <v>163</v>
       </c>
+      <c r="H4" t="s">
+        <v>155</v>
+      </c>
       <c r="I4" s="4" t="s">
         <v>212</v>
       </c>
@@ -1245,6 +1279,9 @@
       <c r="G5" t="s">
         <v>161</v>
       </c>
+      <c r="H5" t="s">
+        <v>155</v>
+      </c>
       <c r="I5" s="4" t="s">
         <v>213</v>
       </c>
@@ -1271,6 +1308,9 @@
       <c r="G6" t="s">
         <v>162</v>
       </c>
+      <c r="H6" t="s">
+        <v>156</v>
+      </c>
       <c r="I6" s="4" t="s">
         <v>214</v>
       </c>
@@ -1297,6 +1337,9 @@
       <c r="G7" t="s">
         <v>162</v>
       </c>
+      <c r="H7" t="s">
+        <v>156</v>
+      </c>
       <c r="I7" s="4" t="s">
         <v>215</v>
       </c>
@@ -1323,6 +1366,9 @@
       <c r="G8" t="s">
         <v>162</v>
       </c>
+      <c r="H8" t="s">
+        <v>156</v>
+      </c>
       <c r="I8" s="4" t="s">
         <v>216</v>
       </c>
@@ -1349,6 +1395,9 @@
       <c r="G9" t="s">
         <v>162</v>
       </c>
+      <c r="H9" t="s">
+        <v>156</v>
+      </c>
       <c r="I9" s="4" t="s">
         <v>225</v>
       </c>
@@ -1375,6 +1424,9 @@
       <c r="G10" t="s">
         <v>162</v>
       </c>
+      <c r="H10" t="s">
+        <v>156</v>
+      </c>
       <c r="I10" s="4" t="s">
         <v>227</v>
       </c>
@@ -1401,6 +1453,9 @@
       <c r="G11" t="s">
         <v>162</v>
       </c>
+      <c r="H11" t="s">
+        <v>156</v>
+      </c>
       <c r="I11" s="4" t="s">
         <v>226</v>
       </c>
@@ -1427,6 +1482,9 @@
       <c r="G12" t="s">
         <v>162</v>
       </c>
+      <c r="H12" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
@@ -1450,6 +1508,9 @@
       <c r="G13" t="s">
         <v>162</v>
       </c>
+      <c r="H13" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -1473,6 +1534,9 @@
       <c r="G14" t="s">
         <v>162</v>
       </c>
+      <c r="H14" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
@@ -1496,6 +1560,9 @@
       <c r="G15" t="s">
         <v>162</v>
       </c>
+      <c r="H15" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
@@ -1519,6 +1586,9 @@
       <c r="G16" t="s">
         <v>162</v>
       </c>
+      <c r="H16" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -1542,6 +1612,9 @@
       <c r="G17" t="s">
         <v>162</v>
       </c>
+      <c r="H17" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18">
@@ -1565,6 +1638,9 @@
       <c r="G18" t="s">
         <v>162</v>
       </c>
+      <c r="H18" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19">
@@ -1588,6 +1664,9 @@
       <c r="G19" t="s">
         <v>162</v>
       </c>
+      <c r="H19" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -1611,6 +1690,9 @@
       <c r="G20" t="s">
         <v>162</v>
       </c>
+      <c r="H20" t="s">
+        <v>156</v>
+      </c>
       <c r="I20" s="5" t="s">
         <v>217</v>
       </c>
@@ -1637,6 +1719,9 @@
       <c r="G21" t="s">
         <v>162</v>
       </c>
+      <c r="H21" t="s">
+        <v>156</v>
+      </c>
       <c r="I21" s="5" t="s">
         <v>218</v>
       </c>
@@ -1663,6 +1748,9 @@
       <c r="G22" t="s">
         <v>162</v>
       </c>
+      <c r="H22" t="s">
+        <v>156</v>
+      </c>
       <c r="I22" s="5" t="s">
         <v>219</v>
       </c>
@@ -1689,6 +1777,9 @@
       <c r="G23" t="s">
         <v>162</v>
       </c>
+      <c r="H23" t="s">
+        <v>156</v>
+      </c>
       <c r="I23" s="5" t="s">
         <v>220</v>
       </c>
@@ -1715,6 +1806,9 @@
       <c r="G24" t="s">
         <v>162</v>
       </c>
+      <c r="H24" t="s">
+        <v>156</v>
+      </c>
       <c r="I24" s="5" t="s">
         <v>228</v>
       </c>
@@ -1741,6 +1835,9 @@
       <c r="G25" t="s">
         <v>162</v>
       </c>
+      <c r="H25" t="s">
+        <v>156</v>
+      </c>
       <c r="I25" s="5" t="s">
         <v>221</v>
       </c>
@@ -1767,6 +1864,9 @@
       <c r="G26" t="s">
         <v>162</v>
       </c>
+      <c r="H26" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27">
@@ -1790,6 +1890,9 @@
       <c r="G27" t="s">
         <v>162</v>
       </c>
+      <c r="H27" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28">
@@ -1813,6 +1916,9 @@
       <c r="G28" t="s">
         <v>162</v>
       </c>
+      <c r="H28" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29">
@@ -1836,6 +1942,9 @@
       <c r="G29" t="s">
         <v>162</v>
       </c>
+      <c r="H29" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30">
@@ -1859,6 +1968,9 @@
       <c r="G30" t="s">
         <v>162</v>
       </c>
+      <c r="H30" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31">
@@ -1882,6 +1994,12 @@
       <c r="G31" t="s">
         <v>162</v>
       </c>
+      <c r="H31" t="s">
+        <v>231</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32">
@@ -1905,8 +2023,14 @@
       <c r="G32" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H32" t="s">
+        <v>231</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>67</v>
       </c>
@@ -1928,8 +2052,14 @@
       <c r="G33" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H33" t="s">
+        <v>231</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4</v>
       </c>
@@ -1951,8 +2081,14 @@
       <c r="G34" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H34" t="s">
+        <v>231</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>20</v>
       </c>
@@ -1974,8 +2110,14 @@
       <c r="G35" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H35" t="s">
+        <v>155</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>69</v>
       </c>
@@ -1997,8 +2139,11 @@
       <c r="G36" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H36" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>-1</v>
       </c>
@@ -2015,7 +2160,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>56</v>
       </c>
@@ -2037,8 +2182,11 @@
       <c r="G38" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H38" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>63</v>
       </c>
@@ -2060,8 +2208,11 @@
       <c r="G39" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H39" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2</v>
       </c>
@@ -2083,8 +2234,11 @@
       <c r="G40" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H40" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>54</v>
       </c>
@@ -2106,8 +2260,11 @@
       <c r="G41" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H41" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>48</v>
       </c>
@@ -2129,8 +2286,11 @@
       <c r="G42" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H42" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>46</v>
       </c>
@@ -2152,8 +2312,11 @@
       <c r="G43" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H43" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>35</v>
       </c>
@@ -2175,8 +2338,11 @@
       <c r="G44" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H44" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>9</v>
       </c>
@@ -2198,8 +2364,11 @@
       <c r="G45" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H45" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>5</v>
       </c>
@@ -2221,8 +2390,11 @@
       <c r="G46" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H46" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>64</v>
       </c>
@@ -2244,8 +2416,11 @@
       <c r="G47" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H47" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>8</v>
       </c>
@@ -2267,8 +2442,11 @@
       <c r="G48" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H48" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>22</v>
       </c>
@@ -2290,8 +2468,11 @@
       <c r="G49" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H49" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>55</v>
       </c>
@@ -2313,8 +2494,11 @@
       <c r="G50" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H50" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>60</v>
       </c>
@@ -2336,8 +2520,11 @@
       <c r="G51" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H51" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>3</v>
       </c>
@@ -2359,8 +2546,11 @@
       <c r="G52" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H52" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>15</v>
       </c>
@@ -2382,8 +2572,11 @@
       <c r="G53" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H53" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>59</v>
       </c>
@@ -2405,8 +2598,11 @@
       <c r="G54" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H54" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>16</v>
       </c>
@@ -2428,8 +2624,11 @@
       <c r="G55" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H55" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>65</v>
       </c>
@@ -2451,8 +2650,11 @@
       <c r="G56" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H56" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>24</v>
       </c>
@@ -2474,8 +2676,11 @@
       <c r="G57" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H57" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>23</v>
       </c>
@@ -2497,8 +2702,11 @@
       <c r="G58" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H58" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>49</v>
       </c>
@@ -2520,8 +2728,11 @@
       <c r="G59" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H59" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>11</v>
       </c>
@@ -2543,8 +2754,11 @@
       <c r="G60" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H60" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>71</v>
       </c>
@@ -2566,8 +2780,11 @@
       <c r="G61" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H61" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>66</v>
       </c>
@@ -2589,8 +2806,11 @@
       <c r="G62" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H62" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>51</v>
       </c>
@@ -2612,8 +2832,11 @@
       <c r="G63" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H63" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>57</v>
       </c>
@@ -2635,8 +2858,11 @@
       <c r="G64" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H64" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>6</v>
       </c>
@@ -2658,8 +2884,11 @@
       <c r="G65" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H65" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>39</v>
       </c>
@@ -2681,8 +2910,11 @@
       <c r="G66" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H66" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>7</v>
       </c>
@@ -2704,8 +2936,11 @@
       <c r="G67" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H67" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>72</v>
       </c>
@@ -2727,8 +2962,11 @@
       <c r="G68" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H68" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>17</v>
       </c>
@@ -2750,8 +2988,11 @@
       <c r="G69" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H69" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>73</v>
       </c>
@@ -2773,8 +3014,11 @@
       <c r="G70" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H70" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>37</v>
       </c>
@@ -2796,8 +3040,11 @@
       <c r="G71" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H71" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>58</v>
       </c>
@@ -2819,8 +3066,11 @@
       <c r="G72" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H72" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>62</v>
       </c>
@@ -2842,8 +3092,11 @@
       <c r="G73" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H73" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>41</v>
       </c>
@@ -2865,8 +3118,11 @@
       <c r="G74" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H74" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>0</v>
       </c>
@@ -2888,8 +3144,11 @@
       <c r="G75" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H75" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>38</v>
       </c>
@@ -2910,6 +3169,9 @@
       </c>
       <c r="G76" t="s">
         <v>162</v>
+      </c>
+      <c r="H76" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -2917,5 +3179,6 @@
     <sortCondition ref="E1:E76"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>